<commit_message>
feat:script test with login and register
</commit_message>
<xml_diff>
--- a/data/data_test2.xlsx
+++ b/data/data_test2.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nam3\KTPM2\Script-test-ecommerece\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learn\Node\Script-test-ecommerece\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E6B200-A12E-47DD-BC7A-ED66D2BD4173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A18B9144-381C-4D38-975F-4180199F9B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Register" sheetId="2" r:id="rId2"/>
+    <sheet name="Register-web" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="116">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -49,9 +50,6 @@
     <t>Expected Result</t>
   </si>
   <si>
-    <t>Actualy result</t>
-  </si>
-  <si>
     <t>Test login with valid credentials</t>
   </si>
   <si>
@@ -160,15 +158,6 @@
     <t>[Login-27]</t>
   </si>
   <si>
-    <t>[Login-28]</t>
-  </si>
-  <si>
-    <t>[Login-29]</t>
-  </si>
-  <si>
-    <t>[Login-30]</t>
-  </si>
-  <si>
     <t>Test login with a password at least 6 character</t>
   </si>
   <si>
@@ -187,9 +176,6 @@
     <t>s</t>
   </si>
   <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
     <t>[Register-8]</t>
   </si>
   <si>
@@ -305,6 +291,99 @@
   </si>
   <si>
     <t>newuser22@example.com</t>
+  </si>
+  <si>
+    <t>Test account registration with valid data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoàng </t>
+  </si>
+  <si>
+    <t>Long</t>
+  </si>
+  <si>
+    <t>long1234@gmail.com</t>
+  </si>
+  <si>
+    <t>Password122</t>
+  </si>
+  <si>
+    <t>Test account registration with an incorrectly formatted email</t>
+  </si>
+  <si>
+    <t>long1234</t>
+  </si>
+  <si>
+    <t>Test account registration with a missing email</t>
+  </si>
+  <si>
+    <t>Test account registration with a missing password</t>
+  </si>
+  <si>
+    <t>Test account registration with both email and password missing</t>
+  </si>
+  <si>
+    <t>Test account registration with an overly long email</t>
+  </si>
+  <si>
+    <t>Password121</t>
+  </si>
+  <si>
+    <t>Test account registration with an overly long password</t>
+  </si>
+  <si>
+    <t>Password122Password122Password122Password122Password122Password122Password122Password122</t>
+  </si>
+  <si>
+    <t>[Register-21]</t>
+  </si>
+  <si>
+    <t>[Register-22]</t>
+  </si>
+  <si>
+    <t>[Register-23]</t>
+  </si>
+  <si>
+    <t>[Register-24]</t>
+  </si>
+  <si>
+    <t>[Register-25]</t>
+  </si>
+  <si>
+    <t>[Register-26]</t>
+  </si>
+  <si>
+    <t>[Register-27]</t>
+  </si>
+  <si>
+    <t>[Login-22]</t>
+  </si>
+  <si>
+    <t>[Login-19]</t>
+  </si>
+  <si>
+    <t>[Login-20]</t>
+  </si>
+  <si>
+    <t>[Login-21]</t>
+  </si>
+  <si>
+    <t>Actual result</t>
+  </si>
+  <si>
+    <t>Password123@</t>
+  </si>
+  <si>
+    <t>Lastname</t>
+  </si>
+  <si>
+    <t>Firstname</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Đà Nẵng</t>
   </si>
 </sst>
 </file>
@@ -410,7 +489,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -584,12 +663,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -643,9 +748,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -703,6 +805,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1039,19 +1162,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>2</v>
@@ -1059,367 +1182,383 @@
     </row>
     <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="40" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="39" t="s">
         <v>14</v>
       </c>
+      <c r="D2" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>13</v>
+      </c>
       <c r="F2" s="16" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="28" t="s">
-        <v>14</v>
+      <c r="D3" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>13</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="6"/>
     </row>
     <row r="4" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="27" t="s">
         <v>14</v>
       </c>
+      <c r="D4" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>13</v>
+      </c>
       <c r="F4" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>14</v>
+        <v>22</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>13</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>14</v>
       </c>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21" t="s">
+        <v>13</v>
+      </c>
       <c r="F6" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="22" t="s">
-        <v>14</v>
+        <v>24</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="21" t="s">
+        <v>13</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="22" t="s">
-        <v>14</v>
+      <c r="D8" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>13</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="F10" s="16"/>
+    <row r="10" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>44</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
+    <row r="11" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
     </row>
     <row r="12" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="7"/>
-      <c r="B12" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="2"/>
+      <c r="A12" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>18</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="C14" s="10"/>
       <c r="D14" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>19</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="D15" s="10"/>
       <c r="E15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="10"/>
+        <v>37</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="D16" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="10"/>
+        <v>28</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="E17" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F17" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>16</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C12" r:id="rId1" xr:uid="{6202DCD7-0689-4C9B-A379-0E93B9037508}"/>
-    <hyperlink ref="C13" r:id="rId2" xr:uid="{CBF8E205-3FC5-4C6D-8D88-984C8782F71C}"/>
-    <hyperlink ref="C14" r:id="rId3" xr:uid="{5C692B60-6AB1-44E2-B091-9578AA47FB33}"/>
-    <hyperlink ref="C15" r:id="rId4" xr:uid="{02DE5336-CF06-4656-BB23-609039868458}"/>
-    <hyperlink ref="C17" r:id="rId5" xr:uid="{4E246B45-84E3-4350-BF34-FE04D281D0E4}"/>
-    <hyperlink ref="C18" r:id="rId6" xr:uid="{5A69D364-3A2F-44E5-B2B8-074A69081BAF}"/>
-    <hyperlink ref="C19" r:id="rId7" xr:uid="{4BE6AA11-F89D-4F5C-BE0A-D662242A7640}"/>
-    <hyperlink ref="C9" r:id="rId8" xr:uid="{147A683F-1E5D-4954-99C7-A4D57833EA90}"/>
-    <hyperlink ref="C2" r:id="rId9" xr:uid="{9A1FA22B-D34F-4D27-B728-47F7F9085B82}"/>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{147A683F-1E5D-4954-99C7-A4D57833EA90}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{9A1FA22B-D34F-4D27-B728-47F7F9085B82}"/>
+    <hyperlink ref="C16" r:id="rId3" xr:uid="{D5DBCD9D-68EB-4C08-B0C7-BCF49DDCA0D6}"/>
+    <hyperlink ref="C10" r:id="rId4" xr:uid="{E6261ACB-45E9-470E-8E97-DA640D50ABBE}"/>
+    <hyperlink ref="D10" r:id="rId5" xr:uid="{E9F4184C-7D12-40ED-8282-9F81B40E960F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -1444,458 +1583,458 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="E1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I1" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I1" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="29" t="s">
+      <c r="J1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="29" t="s">
+      <c r="K1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="29" t="s">
-        <v>50</v>
+      <c r="L1" s="28" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>64</v>
+        <v>67</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>59</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E2" s="2">
         <v>1234567890</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J2" s="16" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="6"/>
     </row>
     <row r="3" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D3" s="38" t="s">
-        <v>67</v>
+        <v>68</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="37" t="s">
+        <v>62</v>
       </c>
       <c r="E3" s="2">
         <v>1234567890</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J3" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="37" t="s">
-        <v>88</v>
+        <v>69</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="D4" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E4" s="2">
         <v>1234567890</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J4" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="38"/>
+        <v>70</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="37"/>
       <c r="E5" s="2">
         <v>1234567890</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J5" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D6" s="37" t="s">
-        <v>88</v>
+        <v>71</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J6" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>88</v>
+        <v>72</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E7" s="2">
         <v>1234567890</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J7" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>88</v>
+        <v>73</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E8" s="2">
         <v>1234567890</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J8" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="37" t="s">
-        <v>88</v>
+        <v>74</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E9" s="2">
         <v>1234567890</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J9" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="6"/>
     </row>
     <row r="10" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="30"/>
-      <c r="D10" s="39"/>
+        <v>75</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="38"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J10" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
     <row r="11" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="37" t="s">
-        <v>88</v>
+        <v>76</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E11" s="2">
         <v>1234567890</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
     <row r="12" spans="1:14" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="36" t="s">
         <v>64</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>69</v>
       </c>
       <c r="E12" s="2">
         <v>1234567890</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J12" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
     <row r="13" spans="1:14" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="36" t="s">
         <v>83</v>
-      </c>
-      <c r="C13" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D13" s="37" t="s">
-        <v>88</v>
       </c>
       <c r="E13" s="2">
         <v>1234567890</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="H13" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J13" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="35" t="s">
-        <v>61</v>
-      </c>
-      <c r="B14" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D14" s="37" t="s">
-        <v>88</v>
+    <row r="14" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="E14" s="2">
         <v>1234567890</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+      <c r="J14" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
     <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="32"/>
+      <c r="A15" s="32"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="31"/>
       <c r="D15" s="10"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -1908,9 +2047,237 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="44" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F16" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G16" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="H16" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K16" s="21"/>
+      <c r="L16" s="21"/>
+    </row>
+    <row r="17" spans="1:12" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="45" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G17" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="H17" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+    </row>
+    <row r="18" spans="1:12" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="45" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" s="41"/>
+      <c r="F18" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G18" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="H18" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+    </row>
+    <row r="19" spans="1:12" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" s="45" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G19" s="43"/>
+      <c r="H19" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+    </row>
+    <row r="20" spans="1:12" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="45" t="s">
+        <v>94</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G20" s="43"/>
+      <c r="H20" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+    </row>
+    <row r="21" spans="1:12" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="B21" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G21" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="H21" s="43"/>
+      <c r="I21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K21" s="21"/>
+      <c r="L21" s="21"/>
+    </row>
+    <row r="22" spans="1:12" ht="97.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E22" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F22" s="41">
+        <v>974791817</v>
+      </c>
+      <c r="G22" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="H22" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K22" s="21"/>
+      <c r="L22" s="21"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C32" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1925,8 +2292,333 @@
     <hyperlink ref="D11" r:id="rId8" xr:uid="{F600AAD8-16AA-4E6E-905B-864335EA3E64}"/>
     <hyperlink ref="D14" r:id="rId9" xr:uid="{5887C2FC-38F8-4A12-A7F5-D8422CCE553E}"/>
     <hyperlink ref="D13" r:id="rId10" xr:uid="{696485C2-177F-4AB4-87E8-EE5BBEB4132E}"/>
+    <hyperlink ref="E16" r:id="rId11" xr:uid="{A4FC3C03-D322-4CCB-A6C8-B647688C34B6}"/>
+    <hyperlink ref="E17" r:id="rId12" display="long1234@gmail.com" xr:uid="{6E1A81D8-9194-456C-A6F1-B0F50576937A}"/>
+    <hyperlink ref="E19" r:id="rId13" xr:uid="{27A7225D-B51E-4890-97A0-C3BB8FA508BF}"/>
+    <hyperlink ref="E21" r:id="rId14" xr:uid="{F4FFCE06-6E88-4377-9692-57FD7EA68064}"/>
+    <hyperlink ref="E22" r:id="rId15" xr:uid="{6C5183ED-9FA7-4AF6-9655-2C0599CFF0D8}"/>
+    <hyperlink ref="G16" r:id="rId16" xr:uid="{0A4AF93A-1A7E-4423-AFE6-55786E24C607}"/>
+    <hyperlink ref="H16" r:id="rId17" xr:uid="{70858BA9-EA56-4F63-8D57-2FB172AC80F7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId18"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3857DA95-2735-4BA6-BAB4-42C63B972C7C}">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" customWidth="1"/>
+    <col min="6" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="J1" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="28" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="28" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G2" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H2" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="I2" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="6"/>
+    </row>
+    <row r="3" spans="1:13" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="45" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G3" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H3" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="I3" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+    </row>
+    <row r="4" spans="1:13" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="45" t="s">
+        <v>92</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H4" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="I4" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+    </row>
+    <row r="5" spans="1:13" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="45" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G5" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+    </row>
+    <row r="6" spans="1:13" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="45" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G6" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G7" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H7" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="I7" s="43"/>
+      <c r="J7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="1:13" ht="166.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="41">
+        <v>8974791817</v>
+      </c>
+      <c r="G8" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="H8" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="I8" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{47AE7072-CE05-4C5F-A063-AEC383335220}"/>
+    <hyperlink ref="E3" r:id="rId2" display="long1234@gmail.com" xr:uid="{A7DBFF08-8DE7-47B4-819D-B6EE1EBD19A6}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{5063378B-8EF3-4200-B2FD-47F715690F38}"/>
+    <hyperlink ref="E7" r:id="rId4" xr:uid="{EF758E16-442C-4175-A3E4-32A1AEA21A5F}"/>
+    <hyperlink ref="E8" r:id="rId5" xr:uid="{A70E0114-7294-4C7A-AE57-A53ACD3435DD}"/>
+    <hyperlink ref="H2" r:id="rId6" xr:uid="{13D9C5B2-BE84-4AEE-9E9B-5E0A401409D6}"/>
+    <hyperlink ref="I2" r:id="rId7" xr:uid="{4EE87AAD-04B6-42CF-BE6C-C091962F8AEB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(app): add new test result files and remove obsolete view.xml
</commit_message>
<xml_diff>
--- a/data/data_test2.xlsx
+++ b/data/data_test2.xlsx
@@ -8,13 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nam3\KTPM2\Script-test-ecommerece\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E6B200-A12E-47DD-BC7A-ED66D2BD4173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E1806B-C91F-4C3F-956D-1327C69B8774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="3360" yWindow="948" windowWidth="17280" windowHeight="8964" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Register" sheetId="2" r:id="rId2"/>
+    <sheet name="Search" sheetId="3" r:id="rId3"/>
+    <sheet name="Cart-web" sheetId="6" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="8" r:id="rId5"/>
+    <sheet name="Search-web" sheetId="7" r:id="rId6"/>
+    <sheet name="Cart" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="219">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -304,7 +309,397 @@
     <t>newusernew@example.com</t>
   </si>
   <si>
-    <t>newuser22@example.com</t>
+    <t>[Cart-11]</t>
+  </si>
+  <si>
+    <t>[Cart-12]</t>
+  </si>
+  <si>
+    <t>[Cart-13]</t>
+  </si>
+  <si>
+    <t>[Cart-14]</t>
+  </si>
+  <si>
+    <t>[Cart-15]</t>
+  </si>
+  <si>
+    <t>[Cart-16]</t>
+  </si>
+  <si>
+    <t>[Cart-17]</t>
+  </si>
+  <si>
+    <t>[Cart-18]</t>
+  </si>
+  <si>
+    <t>[Cart-19]</t>
+  </si>
+  <si>
+    <t>Check view Empty Cart</t>
+  </si>
+  <si>
+    <t>Check redirect from Empty Cart</t>
+  </si>
+  <si>
+    <t>Check add product to cart</t>
+  </si>
+  <si>
+    <t>Check add Same Product Again</t>
+  </si>
+  <si>
+    <t>Check update Cart Product Quantity</t>
+  </si>
+  <si>
+    <t>Check select Single Cart Product</t>
+  </si>
+  <si>
+    <t>Check set Cart Quantity to Zero</t>
+  </si>
+  <si>
+    <t>Check clear All Cart Products</t>
+  </si>
+  <si>
+    <t>Search for a valid product</t>
+  </si>
+  <si>
+    <t>Search with a numeric-only keyword</t>
+  </si>
+  <si>
+    <t>Search for products by valid category</t>
+  </si>
+  <si>
+    <t>Search combining category and keyword</t>
+  </si>
+  <si>
+    <t>Search with a non-existent keyword</t>
+  </si>
+  <si>
+    <t>Search with a short keyword (1 character)</t>
+  </si>
+  <si>
+    <t>Search with a keyword containing spaces</t>
+  </si>
+  <si>
+    <t>Search with special characters</t>
+  </si>
+  <si>
+    <t>Search for a category with no products</t>
+  </si>
+  <si>
+    <t>Search with rapid category switching</t>
+  </si>
+  <si>
+    <t>[Search-12]</t>
+  </si>
+  <si>
+    <t>[Search-13]</t>
+  </si>
+  <si>
+    <t>[Search-14]</t>
+  </si>
+  <si>
+    <t>[Search-15]</t>
+  </si>
+  <si>
+    <t>[Search-16]</t>
+  </si>
+  <si>
+    <t>[Search-17]</t>
+  </si>
+  <si>
+    <t>[Search-18]</t>
+  </si>
+  <si>
+    <t>[Search-19]</t>
+  </si>
+  <si>
+    <t>[Search-20]</t>
+  </si>
+  <si>
+    <t>[Search-21]</t>
+  </si>
+  <si>
+    <t>Key Words</t>
+  </si>
+  <si>
+    <t>iPhone 13</t>
+  </si>
+  <si>
+    <t>Displays a list of products related to "iPhone 13".</t>
+  </si>
+  <si>
+    <t>Displays a list of products related to items containing "13".</t>
+  </si>
+  <si>
+    <t>Displays a list of all products in the "iPhone" category.</t>
+  </si>
+  <si>
+    <t>Displays all available products.</t>
+  </si>
+  <si>
+    <t>Displays all products with names containing "a".</t>
+  </si>
+  <si>
+    <t>Displays a message: "No products found".</t>
+  </si>
+  <si>
+    <t>Displays a list of products in the "Samsung" category.</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>i Phone 13</t>
+  </si>
+  <si>
+    <t>"@#$%"</t>
+  </si>
+  <si>
+    <t>- A message is displayed: "Your cart is empty".</t>
+  </si>
+  <si>
+    <t>- The total price is updated based on the selected product.</t>
+  </si>
+  <si>
+    <t>- All products are removed from the cart.
+- A message is displayed: "Your cart is empty".</t>
+  </si>
+  <si>
+    <t>- The application redirects to the Home Screen.</t>
+  </si>
+  <si>
+    <t>newuser27@example.com</t>
+  </si>
+  <si>
+    <t>- Displays a message: "Added to cart".
+- "iPhone 13" and "Samsung Galaxy S24 FE 5G" appears in the cart with a quantity of 1</t>
+  </si>
+  <si>
+    <t>- Quantity of "Samsung Galaxy S24 FE 5G" in the cart increases to 2.- Total price updates correctly.</t>
+  </si>
+  <si>
+    <t>Check update Large Product Quantity</t>
+  </si>
+  <si>
+    <t>Check select All Cart Product</t>
+  </si>
+  <si>
+    <t>- The quantity of "Samsung Galaxy S24 FE 5G" is updated to 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- The "iPhone 13" product has a quantity of 10 in the cart.
+</t>
+  </si>
+  <si>
+    <t>- The total price is updated based on the all product.</t>
+  </si>
+  <si>
+    <t>- The Quantity of "iPhone 13" to One.</t>
+  </si>
+  <si>
+    <t>[Cart-20]</t>
+  </si>
+  <si>
+    <t>Displays a list of "Galaxy S24" products within the "Samsung" category.</t>
+  </si>
+  <si>
+    <t>Galaxy S24</t>
+  </si>
+  <si>
+    <t>Actual result</t>
+  </si>
+  <si>
+    <t>[Login-20]</t>
+  </si>
+  <si>
+    <t>Test adding a product to the cart</t>
+  </si>
+  <si>
+    <t>hoanglong2007032@gmail.com</t>
+  </si>
+  <si>
+    <t>Tgdt1234@</t>
+  </si>
+  <si>
+    <t>Cart displays the selected product, quantity 1</t>
+  </si>
+  <si>
+    <t>[Login-21]</t>
+  </si>
+  <si>
+    <t>Test viewing cart contents</t>
+  </si>
+  <si>
+    <t>[Login-22]</t>
+  </si>
+  <si>
+    <t>Test increasing product quantity</t>
+  </si>
+  <si>
+    <t>Quantity increases to 2, total price updates accordingly</t>
+  </si>
+  <si>
+    <t>Test calculating total amount in cart</t>
+  </si>
+  <si>
+    <t>Total amount reflects the product's price and quantity</t>
+  </si>
+  <si>
+    <t>Test removing a product from the cart</t>
+  </si>
+  <si>
+    <t>Message: "Deleted product successful", cart empty</t>
+  </si>
+  <si>
+    <t>Test adding the same product multiple times</t>
+  </si>
+  <si>
+    <t>Selected product quantity 2</t>
+  </si>
+  <si>
+    <t>Test checkout with an empty cart</t>
+  </si>
+  <si>
+    <t>Cart retains the selected product, quantity 1</t>
+  </si>
+  <si>
+    <t>Test add products to cart after login</t>
+  </si>
+  <si>
+    <t>Cart displays the selected product</t>
+  </si>
+  <si>
+    <t>Test product quantity reduction</t>
+  </si>
+  <si>
+    <t>Quantity decreases to 1, total price updates; if 0, "Your cart is empty"</t>
+  </si>
+  <si>
+    <t>Test add products to cart before login</t>
+  </si>
+  <si>
+    <t>Redirect to login page</t>
+  </si>
+  <si>
+    <t>SearchQuery</t>
+  </si>
+  <si>
+    <t>Search for a valid product by name</t>
+  </si>
+  <si>
+    <t>samsung</t>
+  </si>
+  <si>
+    <t>Products found</t>
+  </si>
+  <si>
+    <t>No products found</t>
+  </si>
+  <si>
+    <t>Case-insensitive search</t>
+  </si>
+  <si>
+    <t>SAMSUNG</t>
+  </si>
+  <si>
+    <t>Search with leading and trailing spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> samsung</t>
+  </si>
+  <si>
+    <t>Search with multiple spaces between words</t>
+  </si>
+  <si>
+    <t>samsung          galaxy</t>
+  </si>
+  <si>
+    <t>[Login-19]</t>
+  </si>
+  <si>
+    <t>Search using numeric keywords</t>
+  </si>
+  <si>
+    <t>#$%</t>
+  </si>
+  <si>
+    <t>Firstname</t>
+  </si>
+  <si>
+    <t>Lastname</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>[Register-21]</t>
+  </si>
+  <si>
+    <t>Test account registration with valid data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoàng </t>
+  </si>
+  <si>
+    <t>Long</t>
+  </si>
+  <si>
+    <t>long1234@gmail.com</t>
+  </si>
+  <si>
+    <t>Đà Nẵng</t>
+  </si>
+  <si>
+    <t>Password123@</t>
+  </si>
+  <si>
+    <t>[Register-22]</t>
+  </si>
+  <si>
+    <t>Test account registration with an incorrectly formatted email</t>
+  </si>
+  <si>
+    <t>long1234</t>
+  </si>
+  <si>
+    <t>Password122</t>
+  </si>
+  <si>
+    <t>[Register-23]</t>
+  </si>
+  <si>
+    <t>Test account registration with a missing email</t>
+  </si>
+  <si>
+    <t>[Register-24]</t>
+  </si>
+  <si>
+    <t>Test account registration with a missing password</t>
+  </si>
+  <si>
+    <t>[Register-25]</t>
+  </si>
+  <si>
+    <t>Test account registration with both email and password missing</t>
+  </si>
+  <si>
+    <t>[Register-26]</t>
+  </si>
+  <si>
+    <t>Test account registration with an overly long email</t>
+  </si>
+  <si>
+    <t>Password121</t>
+  </si>
+  <si>
+    <t>[Register-27]</t>
+  </si>
+  <si>
+    <t>Test account registration with an overly long password</t>
+  </si>
+  <si>
+    <t>Password122Password122Password122Password122Password122Password122Password122Password122</t>
   </si>
 </sst>
 </file>
@@ -410,7 +805,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -584,12 +979,64 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -703,6 +1150,57 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1485,7 +1983,7 @@
         <v>64</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>89</v>
+        <v>142</v>
       </c>
       <c r="E2" s="2">
         <v>1234567890</v>
@@ -1929,4 +2427,1227 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33F4662B-82A0-46A1-98AD-114073110E2E}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" spans="1:7" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" s="22">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="46" t="s">
+        <v>129</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="6"/>
+    </row>
+    <row r="5" spans="1:7" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="46" t="s">
+        <v>152</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="6"/>
+    </row>
+    <row r="6" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="22"/>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="6"/>
+    </row>
+    <row r="8" spans="1:7" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="6"/>
+    </row>
+    <row r="9" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDAE0FF7-C004-47C8-A231-364ED16C00E3}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="30.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="30.77734375" style="52"/>
+    <col min="5" max="5" width="46.21875" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" customWidth="1"/>
+    <col min="7" max="7" width="28.77734375" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
+    <col min="9" max="9" width="6.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="H1" s="47" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="50"/>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="48" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="50"/>
+    </row>
+    <row r="4" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="42" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="51"/>
+    </row>
+    <row r="5" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="42" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="51"/>
+    </row>
+    <row r="6" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="51"/>
+    </row>
+    <row r="7" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="48" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="51"/>
+    </row>
+    <row r="8" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="51"/>
+    </row>
+    <row r="9" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="48" t="s">
+        <v>173</v>
+      </c>
+      <c r="C9" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="51"/>
+    </row>
+    <row r="10" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="48" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="51"/>
+    </row>
+    <row r="11" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="48" t="s">
+        <v>177</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="51"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C12"/>
+      <c r="D12"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{64F61CCD-F607-4DE1-8EAE-D50D5FB4D4F4}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{9E3A3E87-9CBE-403C-9078-D0742ADB805F}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{CECEE67D-E731-46AF-A981-2BD5C5473FFD}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{199B8B0F-B7F2-47A1-9BD7-AD1E672B2AD5}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{1D089417-FAA3-4587-A5B1-45A526E18B1D}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{6B1F26A3-817D-4FEF-90CA-C6FD894F64A4}"/>
+    <hyperlink ref="C8" r:id="rId7" xr:uid="{3D89C201-1833-49CB-AB26-A829431203C7}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{BAB88D17-84E9-4C11-9D36-F5389B8CFE13}"/>
+    <hyperlink ref="C10" r:id="rId9" xr:uid="{38926D84-A229-43E9-AFB3-79E8A022B1EF}"/>
+    <hyperlink ref="C11" r:id="rId10" xr:uid="{F2BF7D3D-68FF-4512-8D18-880601D33B93}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{778C1D54-C53D-48D4-AC46-61838858D02E}">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultColWidth="15.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:13" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" s="41" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="29" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="42" t="s">
+        <v>196</v>
+      </c>
+      <c r="B2" s="53" t="s">
+        <v>197</v>
+      </c>
+      <c r="C2" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D2" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E2" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="F2" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G2" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H2" s="56" t="s">
+        <v>202</v>
+      </c>
+      <c r="I2" s="56" t="s">
+        <v>202</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="6"/>
+    </row>
+    <row r="3" spans="1:13" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="42" t="s">
+        <v>203</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="C3" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D3" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E3" s="55" t="s">
+        <v>205</v>
+      </c>
+      <c r="F3" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G3" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H3" s="58" t="s">
+        <v>206</v>
+      </c>
+      <c r="I3" s="58" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+    </row>
+    <row r="4" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="42" t="s">
+        <v>207</v>
+      </c>
+      <c r="B4" s="57" t="s">
+        <v>208</v>
+      </c>
+      <c r="C4" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G4" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H4" s="58" t="s">
+        <v>206</v>
+      </c>
+      <c r="I4" s="58" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+    </row>
+    <row r="5" spans="1:13" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="42" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="C5" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E5" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="F5" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G5" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+    </row>
+    <row r="6" spans="1:13" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="42" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" s="57" t="s">
+        <v>212</v>
+      </c>
+      <c r="C6" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D6" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G6" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H6" s="58"/>
+      <c r="I6" s="58" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="42" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="57" t="s">
+        <v>214</v>
+      </c>
+      <c r="C7" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D7" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E7" s="55" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G7" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H7" s="58" t="s">
+        <v>215</v>
+      </c>
+      <c r="I7" s="58"/>
+      <c r="J7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="1:13" ht="97.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="42" t="s">
+        <v>216</v>
+      </c>
+      <c r="B8" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="C8" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E8" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="F8" s="54">
+        <v>8974791817</v>
+      </c>
+      <c r="G8" s="54" t="s">
+        <v>201</v>
+      </c>
+      <c r="H8" s="58" t="s">
+        <v>218</v>
+      </c>
+      <c r="I8" s="58" t="s">
+        <v>218</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{CD49152F-D1FF-4D79-A8E0-0750CAD4B180}"/>
+    <hyperlink ref="E3" r:id="rId2" display="long1234@gmail.com" xr:uid="{7022E786-974D-4D7B-8F12-23D1F6D7205F}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{899F5B40-87DC-48E7-AD59-9E599766D790}"/>
+    <hyperlink ref="E7" r:id="rId4" xr:uid="{F6614410-E1A5-47AE-88E1-0EC10CB9809D}"/>
+    <hyperlink ref="E8" r:id="rId5" xr:uid="{A0CC158E-83D9-4CD4-B295-9004E234BD4C}"/>
+    <hyperlink ref="H2" r:id="rId6" xr:uid="{85C044DC-0106-463A-B3C6-EE86228F7E70}"/>
+    <hyperlink ref="I2" r:id="rId7" xr:uid="{F9F70111-5AC6-4D99-9F62-31B7A028653E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1867D617-8DB4-4D75-9F59-9BCE8AF7A9D2}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G1" s="47" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+      <c r="A2" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="50"/>
+    </row>
+    <row r="3" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+      <c r="A3" s="42" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="50"/>
+    </row>
+    <row r="4" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="42" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="43" t="s">
+        <v>184</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="51"/>
+    </row>
+    <row r="5" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="51"/>
+    </row>
+    <row r="6" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="43" t="s">
+        <v>188</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="51"/>
+    </row>
+    <row r="7" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+      <c r="A7" s="42" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" s="43" t="s">
+        <v>191</v>
+      </c>
+      <c r="C7" s="10">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="51"/>
+    </row>
+    <row r="8" spans="1:7" ht="96.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="51"/>
+    </row>
+    <row r="9" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+      <c r="A9" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="51"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74705681-7C46-484E-AF9C-A55FF07C4166}">
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.5546875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="21.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="42" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" ht="97.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="46" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="42" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>147</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="42" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>145</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>139</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>149</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="44" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>150</v>
+      </c>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+    </row>
+    <row r="11" spans="1:8" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="44" t="s">
+        <v>151</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="42"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(app): update test result files for cart, search, and data_test2
</commit_message>
<xml_diff>
--- a/data/data_test2.xlsx
+++ b/data/data_test2.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nam3\KTPM2\Script-test-ecommerece\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E1806B-C91F-4C3F-956D-1327C69B8774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E358F650-700D-4B32-8CCF-27436DE1B12D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="948" windowWidth="17280" windowHeight="8964" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Register" sheetId="2" r:id="rId2"/>
     <sheet name="Search" sheetId="3" r:id="rId3"/>
     <sheet name="Cart-web" sheetId="6" r:id="rId4"/>
-    <sheet name="Sheet3" sheetId="8" r:id="rId5"/>
+    <sheet name="Register_web" sheetId="8" r:id="rId5"/>
     <sheet name="Search-web" sheetId="7" r:id="rId6"/>
     <sheet name="Cart" sheetId="5" r:id="rId7"/>
   </sheets>

</xml_diff>

<commit_message>
feat(data): update data_test2.xlsx file
</commit_message>
<xml_diff>
--- a/data/data_test2.xlsx
+++ b/data/data_test2.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nam3\KTPM2\Script-test-ecommerece\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Test\script-test\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E1806B-C91F-4C3F-956D-1327C69B8774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C163C8F-E1C6-406A-94C5-95A7D15B2AAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="948" windowWidth="17280" windowHeight="8964" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="4" xr2:uid="{8FAFAB84-7321-4A60-AD43-F6BDBFF31D96}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Register" sheetId="2" r:id="rId2"/>
     <sheet name="Search" sheetId="3" r:id="rId3"/>
     <sheet name="Cart-web" sheetId="6" r:id="rId4"/>
-    <sheet name="Sheet3" sheetId="8" r:id="rId5"/>
+    <sheet name="Register_web" sheetId="8" r:id="rId5"/>
     <sheet name="Search-web" sheetId="7" r:id="rId6"/>
     <sheet name="Cart" sheetId="5" r:id="rId7"/>
   </sheets>
@@ -1518,18 +1518,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A869C040-2518-4127-9479-80AA9CA67B0C}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="35.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>20</v>
       </c>
@@ -1577,7 +1577,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>21</v>
       </c>
@@ -1599,7 +1599,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>22</v>
       </c>
@@ -1621,7 +1621,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
         <v>23</v>
       </c>
@@ -1641,7 +1641,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>24</v>
       </c>
@@ -1661,7 +1661,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>25</v>
       </c>
@@ -1679,7 +1679,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
         <v>26</v>
       </c>
@@ -1701,7 +1701,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
         <v>27</v>
       </c>
@@ -1723,17 +1723,17 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="F10" s="16"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F11" s="23"/>
       <c r="G11" s="23"/>
       <c r="H11" s="23"/>
     </row>
-    <row r="12" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
       <c r="B12" s="17" t="s">
         <v>5</v>
@@ -1751,7 +1751,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>36</v>
       </c>
@@ -1771,7 +1771,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>37</v>
       </c>
@@ -1791,7 +1791,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>38</v>
       </c>
@@ -1811,7 +1811,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>39</v>
       </c>
@@ -1829,7 +1829,7 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>40</v>
       </c>
@@ -1847,7 +1847,7 @@
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>41</v>
       </c>
@@ -1867,7 +1867,7 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>42</v>
       </c>
@@ -1887,7 +1887,7 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>43</v>
       </c>
@@ -1924,17 +1924,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEC2713A-74A1-4D69-BE27-025D72CC84F9}">
   <dimension ref="A1:N32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="7" width="14.88671875" customWidth="1"/>
+    <col min="5" max="7" width="14.85546875" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>51</v>
       </c>
@@ -2006,7 +2006,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="6"/>
     </row>
-    <row r="3" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>52</v>
       </c>
@@ -2040,7 +2040,7 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>53</v>
       </c>
@@ -2072,7 +2072,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>54</v>
       </c>
@@ -2104,7 +2104,7 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>55</v>
       </c>
@@ -2136,7 +2136,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>56</v>
       </c>
@@ -2168,7 +2168,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>57</v>
       </c>
@@ -2200,7 +2200,7 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>58</v>
       </c>
@@ -2232,7 +2232,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="6"/>
     </row>
-    <row r="10" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>59</v>
       </c>
@@ -2254,7 +2254,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>62</v>
       </c>
@@ -2288,7 +2288,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:14" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>63</v>
       </c>
@@ -2322,7 +2322,7 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:14" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>60</v>
       </c>
@@ -2356,7 +2356,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A14" s="35" t="s">
         <v>61</v>
       </c>
@@ -2390,7 +2390,7 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="33"/>
       <c r="B15" s="34"/>
       <c r="C15" s="32"/>
@@ -2406,7 +2406,7 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C32" t="s">
         <v>49</v>
       </c>
@@ -2432,15 +2432,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33F4662B-82A0-46A1-98AD-114073110E2E}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>116</v>
       </c>
@@ -2482,7 +2482,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="1:7" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>117</v>
       </c>
@@ -2501,7 +2501,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>118</v>
       </c>
@@ -2518,7 +2518,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="6"/>
     </row>
-    <row r="5" spans="1:7" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>119</v>
       </c>
@@ -2537,7 +2537,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>120</v>
       </c>
@@ -2554,7 +2554,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="6"/>
     </row>
-    <row r="7" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>121</v>
       </c>
@@ -2573,7 +2573,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" spans="1:7" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>122</v>
       </c>
@@ -2592,7 +2592,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="6"/>
     </row>
-    <row r="9" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>123</v>
       </c>
@@ -2611,7 +2611,7 @@
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
     </row>
-    <row r="10" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>124</v>
       </c>
@@ -2628,7 +2628,7 @@
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
     </row>
-    <row r="11" spans="1:7" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>125</v>
       </c>
@@ -2654,18 +2654,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDAE0FF7-C004-47C8-A231-364ED16C00E3}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="30.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="30.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="30.77734375" style="52"/>
-    <col min="5" max="5" width="46.21875" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" customWidth="1"/>
-    <col min="7" max="7" width="28.77734375" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="30.7109375" style="52"/>
+    <col min="5" max="5" width="46.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="28.7109375" customWidth="1"/>
     <col min="8" max="8" width="38" customWidth="1"/>
-    <col min="9" max="9" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2691,7 +2691,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>155</v>
       </c>
@@ -2713,7 +2713,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="50"/>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
         <v>160</v>
       </c>
@@ -2735,7 +2735,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="50"/>
     </row>
-    <row r="4" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="42" t="s">
         <v>162</v>
       </c>
@@ -2757,7 +2757,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="51"/>
     </row>
-    <row r="5" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="42" t="s">
         <v>36</v>
       </c>
@@ -2779,7 +2779,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="51"/>
     </row>
-    <row r="6" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="42" t="s">
         <v>37</v>
       </c>
@@ -2801,7 +2801,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="51"/>
     </row>
-    <row r="7" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
         <v>38</v>
       </c>
@@ -2823,7 +2823,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="51"/>
     </row>
-    <row r="8" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="42" t="s">
         <v>39</v>
       </c>
@@ -2845,7 +2845,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="51"/>
     </row>
-    <row r="9" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
         <v>40</v>
       </c>
@@ -2867,7 +2867,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="51"/>
     </row>
-    <row r="10" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="42" t="s">
         <v>41</v>
       </c>
@@ -2889,7 +2889,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="51"/>
     </row>
-    <row r="11" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A11" s="42" t="s">
         <v>42</v>
       </c>
@@ -2911,7 +2911,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="51"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C12"/>
       <c r="D12"/>
     </row>
@@ -2935,9 +2935,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{778C1D54-C53D-48D4-AC46-61838858D02E}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultColWidth="15.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2978,7 +2978,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="s">
         <v>196</v>
       </c>
@@ -3015,7 +3015,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="6"/>
     </row>
-    <row r="3" spans="1:13" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="42" t="s">
         <v>203</v>
       </c>
@@ -3052,7 +3052,7 @@
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:13" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="42" t="s">
         <v>207</v>
       </c>
@@ -3087,7 +3087,7 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="42" t="s">
         <v>209</v>
       </c>
@@ -3122,7 +3122,7 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="42" t="s">
         <v>211</v>
       </c>
@@ -3155,7 +3155,7 @@
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="1:13" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="42" t="s">
         <v>213</v>
       </c>
@@ -3190,7 +3190,7 @@
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13" ht="97.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="42" t="s">
         <v>216</v>
       </c>
@@ -3244,9 +3244,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1867D617-8DB4-4D75-9F59-9BCE8AF7A9D2}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="57" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3269,7 +3269,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>23</v>
       </c>
@@ -3288,7 +3288,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="50"/>
     </row>
-    <row r="3" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
         <v>24</v>
       </c>
@@ -3305,7 +3305,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="50"/>
     </row>
-    <row r="4" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A4" s="42" t="s">
         <v>25</v>
       </c>
@@ -3324,7 +3324,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="51"/>
     </row>
-    <row r="5" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A5" s="42" t="s">
         <v>26</v>
       </c>
@@ -3343,7 +3343,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="51"/>
     </row>
-    <row r="6" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="85.5" x14ac:dyDescent="0.25">
       <c r="A6" s="42" t="s">
         <v>27</v>
       </c>
@@ -3362,7 +3362,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="51"/>
     </row>
-    <row r="7" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
         <v>190</v>
       </c>
@@ -3381,7 +3381,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="51"/>
     </row>
-    <row r="8" spans="1:7" ht="96.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A8" s="42" t="s">
         <v>155</v>
       </c>
@@ -3400,7 +3400,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="51"/>
     </row>
-    <row r="9" spans="1:7" ht="69" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
         <v>155</v>
       </c>
@@ -3427,14 +3427,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74705681-7C46-484E-AF9C-A55FF07C4166}">
   <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="21.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="s">
         <v>89</v>
       </c>
@@ -3470,7 +3470,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="42" t="s">
         <v>90</v>
       </c>
@@ -3486,7 +3486,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" spans="1:8" ht="97.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="114.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="42" t="s">
         <v>91</v>
       </c>
@@ -3502,7 +3502,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="6"/>
     </row>
-    <row r="5" spans="1:8" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="42" t="s">
         <v>92</v>
       </c>
@@ -3518,7 +3518,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="6"/>
     </row>
-    <row r="6" spans="1:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="42" t="s">
         <v>93</v>
       </c>
@@ -3534,7 +3534,7 @@
       <c r="E6" s="2"/>
       <c r="F6" s="6"/>
     </row>
-    <row r="7" spans="1:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="42" t="s">
         <v>94</v>
       </c>
@@ -3550,7 +3550,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="6"/>
     </row>
-    <row r="8" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="42" t="s">
         <v>95</v>
       </c>
@@ -3566,7 +3566,7 @@
       <c r="E8" s="2"/>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="42" t="s">
         <v>96</v>
       </c>
@@ -3582,7 +3582,7 @@
       <c r="E9" s="2"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="44" t="s">
         <v>97</v>
       </c>
@@ -3598,7 +3598,7 @@
       <c r="E10" s="45"/>
       <c r="F10" s="45"/>
     </row>
-    <row r="11" spans="1:8" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="44" t="s">
         <v>151</v>
       </c>
@@ -3616,7 +3616,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="6"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="42"/>
       <c r="B12" s="43"/>
       <c r="C12" s="22"/>
@@ -3626,7 +3626,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="6"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="42"/>
       <c r="B13" s="43"/>
       <c r="C13" s="22"/>
@@ -3636,7 +3636,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="6"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="42"/>
       <c r="B14" s="43"/>
       <c r="C14" s="22"/>

</xml_diff>